<commit_message>
drop the pipeline image link until the diagram is redrawn for the new layout
</commit_message>
<xml_diff>
--- a/05_Figures/HRvLR/F2_Programmes/c_data/f2_programmes.xlsx
+++ b/05_Figures/HRvLR/F2_Programmes/c_data/f2_programmes.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1256" uniqueCount="317">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1289" uniqueCount="338">
   <si>
     <t>sheet</t>
   </si>
@@ -291,7 +291,7 @@
     <t>eigengene logFC and evidence, fry evidence</t>
   </si>
   <si>
-    <t>02_HRvLR_groups/04_Module_Contrasts/c_data/module_contrasts.xlsx</t>
+    <t>03_Group_comparisons/HRvLR/04_Module_Contrasts/c_data/module_contrasts.xlsx</t>
   </si>
   <si>
     <t>eigengene_tests, fry_tests</t>
@@ -306,7 +306,7 @@
     <t>sets called per contrast</t>
   </si>
   <si>
-    <t>02_HRvLR_groups/03_Set_Contrasts/c_data/set_tests.rds</t>
+    <t>03_Group_comparisons/HRvLR/03_Set_Contrasts/c_data/set_tests.rds</t>
   </si>
   <si>
     <t>set_tests</t>
@@ -582,16 +582,16 @@
     <t>design</t>
   </si>
   <si>
-    <t>02_HRvLR_groups/01_Design_Contrasts/c_data/design_contrasts.xlsx</t>
-  </si>
-  <si>
-    <t>39540089eab402ee5a70d7765367711f</t>
+    <t>03_Group_comparisons/HRvLR/01_Design_Contrasts/c_data/design_contrasts.xlsx</t>
+  </si>
+  <si>
+    <t>ba6f06ab566bcd628808d4bba0453ec3</t>
   </si>
   <si>
     <t>module_tests</t>
   </si>
   <si>
-    <t>d34ea4613b20d81703717017a28b09a7</t>
+    <t>ecbb45481c166acd896958a6dea708c1</t>
   </si>
   <si>
     <t>b928dfb75f0631b92e8ffaf819778f86</t>
@@ -600,10 +600,10 @@
     <t>set_summary</t>
   </si>
   <si>
-    <t>02_HRvLR_groups/03_Set_Contrasts/c_data/set_contrasts.xlsx</t>
-  </si>
-  <si>
-    <t>4881d4307de24d7bff3c51428ffaaf37</t>
+    <t>03_Group_comparisons/HRvLR/03_Set_Contrasts/c_data/set_contrasts.xlsx</t>
+  </si>
+  <si>
+    <t>32b8e3d423a3c1ea391dcc422f505b2e</t>
   </si>
   <si>
     <t>modules</t>
@@ -615,7 +615,7 @@
     <t>module_labels</t>
   </si>
   <si>
-    <t>218ea5b0a99df49bcf01bd7e91c02753</t>
+    <t>2d44b6abe30000872e9818e6c5763c8b</t>
   </si>
   <si>
     <t>BiocGenerics</t>
@@ -720,12 +720,24 @@
     <t>1.2.1</t>
   </si>
   <si>
+    <t>evaluate</t>
+  </si>
+  <si>
+    <t>1.0.5</t>
+  </si>
+  <si>
     <t>farver</t>
   </si>
   <si>
     <t>2.1.2</t>
   </si>
   <si>
+    <t>fastmap</t>
+  </si>
+  <si>
+    <t>1.2.0</t>
+  </si>
+  <si>
     <t>foreach</t>
   </si>
   <si>
@@ -783,6 +795,18 @@
     <t>1.1.4</t>
   </si>
   <si>
+    <t>htmltools</t>
+  </si>
+  <si>
+    <t>0.5.9</t>
+  </si>
+  <si>
+    <t>htmlwidgets</t>
+  </si>
+  <si>
+    <t>1.6.4</t>
+  </si>
+  <si>
     <t>IRanges</t>
   </si>
   <si>
@@ -795,6 +819,18 @@
     <t>1.0.14</t>
   </si>
   <si>
+    <t>jsonlite</t>
+  </si>
+  <si>
+    <t>2.0.0</t>
+  </si>
+  <si>
+    <t>knitr</t>
+  </si>
+  <si>
+    <t>1.51</t>
+  </si>
+  <si>
     <t>labeling</t>
   </si>
   <si>
@@ -804,9 +840,6 @@
     <t>lifecycle</t>
   </si>
   <si>
-    <t>1.0.5</t>
-  </si>
-  <si>
     <t>magrittr</t>
   </si>
   <si>
@@ -819,6 +852,12 @@
     <t>1.5.0</t>
   </si>
   <si>
+    <t>otel</t>
+  </si>
+  <si>
+    <t>0.2.0</t>
+  </si>
+  <si>
     <t>patchwork</t>
   </si>
   <si>
@@ -894,6 +933,12 @@
     <t>CRAN (R 4.6.1)</t>
   </si>
   <si>
+    <t>rmarkdown</t>
+  </si>
+  <si>
+    <t>2.31</t>
+  </si>
+  <si>
     <t>rprojroot</t>
   </si>
   <si>
@@ -960,6 +1005,12 @@
     <t>0.5.0</t>
   </si>
   <si>
+    <t>utf8</t>
+  </si>
+  <si>
+    <t>1.2.6</t>
+  </si>
+  <si>
     <t>vctrs</t>
   </si>
   <si>
@@ -976,6 +1027,18 @@
   </si>
   <si>
     <t>3.0.2</t>
+  </si>
+  <si>
+    <t>xfun</t>
+  </si>
+  <si>
+    <t>0.57</t>
+  </si>
+  <si>
+    <t>yaml</t>
+  </si>
+  <si>
+    <t>2.3.12</t>
   </si>
 </sst>
 </file>
@@ -7561,7 +7624,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C61"/>
+  <dimension ref="A1:C72"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
@@ -7822,7 +7885,7 @@
         <v>243</v>
       </c>
       <c r="B24" t="s">
-        <v>236</v>
+        <v>244</v>
       </c>
       <c r="C24" t="s">
         <v>202</v>
@@ -7830,10 +7893,10 @@
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B25" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C25" t="s">
         <v>202</v>
@@ -7841,10 +7904,10 @@
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="B26" t="s">
-        <v>247</v>
+        <v>240</v>
       </c>
       <c r="C26" t="s">
         <v>202</v>
@@ -7880,7 +7943,7 @@
         <v>253</v>
       </c>
       <c r="C29" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
     </row>
     <row r="30" spans="1:3">
@@ -7924,7 +7987,7 @@
         <v>261</v>
       </c>
       <c r="C33" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
     </row>
     <row r="34" spans="1:3">
@@ -7976,7 +8039,7 @@
         <v>270</v>
       </c>
       <c r="B38" t="s">
-        <v>271</v>
+        <v>232</v>
       </c>
       <c r="C38" t="s">
         <v>202</v>
@@ -7984,10 +8047,10 @@
     </row>
     <row r="39" spans="1:3">
       <c r="A39" t="s">
+        <v>271</v>
+      </c>
+      <c r="B39" t="s">
         <v>272</v>
-      </c>
-      <c r="B39" t="s">
-        <v>273</v>
       </c>
       <c r="C39" t="s">
         <v>202</v>
@@ -7995,10 +8058,10 @@
     </row>
     <row r="40" spans="1:3">
       <c r="A40" t="s">
+        <v>273</v>
+      </c>
+      <c r="B40" t="s">
         <v>274</v>
-      </c>
-      <c r="B40" t="s">
-        <v>275</v>
       </c>
       <c r="C40" t="s">
         <v>202</v>
@@ -8006,10 +8069,10 @@
     </row>
     <row r="41" spans="1:3">
       <c r="A41" t="s">
+        <v>275</v>
+      </c>
+      <c r="B41" t="s">
         <v>276</v>
-      </c>
-      <c r="B41" t="s">
-        <v>277</v>
       </c>
       <c r="C41" t="s">
         <v>202</v>
@@ -8017,10 +8080,10 @@
     </row>
     <row r="42" spans="1:3">
       <c r="A42" t="s">
+        <v>277</v>
+      </c>
+      <c r="B42" t="s">
         <v>278</v>
-      </c>
-      <c r="B42" t="s">
-        <v>279</v>
       </c>
       <c r="C42" t="s">
         <v>202</v>
@@ -8028,10 +8091,10 @@
     </row>
     <row r="43" spans="1:3">
       <c r="A43" t="s">
+        <v>279</v>
+      </c>
+      <c r="B43" t="s">
         <v>280</v>
-      </c>
-      <c r="B43" t="s">
-        <v>281</v>
       </c>
       <c r="C43" t="s">
         <v>202</v>
@@ -8039,10 +8102,10 @@
     </row>
     <row r="44" spans="1:3">
       <c r="A44" t="s">
+        <v>281</v>
+      </c>
+      <c r="B44" t="s">
         <v>282</v>
-      </c>
-      <c r="B44" t="s">
-        <v>283</v>
       </c>
       <c r="C44" t="s">
         <v>202</v>
@@ -8050,10 +8113,10 @@
     </row>
     <row r="45" spans="1:3">
       <c r="A45" t="s">
+        <v>283</v>
+      </c>
+      <c r="B45" t="s">
         <v>284</v>
-      </c>
-      <c r="B45" t="s">
-        <v>285</v>
       </c>
       <c r="C45" t="s">
         <v>202</v>
@@ -8061,21 +8124,21 @@
     </row>
     <row r="46" spans="1:3">
       <c r="A46" t="s">
+        <v>285</v>
+      </c>
+      <c r="B46" t="s">
         <v>286</v>
       </c>
-      <c r="B46" t="s">
-        <v>287</v>
-      </c>
       <c r="C46" t="s">
-        <v>288</v>
+        <v>202</v>
       </c>
     </row>
     <row r="47" spans="1:3">
       <c r="A47" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="B47" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="C47" t="s">
         <v>202</v>
@@ -8083,21 +8146,21 @@
     </row>
     <row r="48" spans="1:3">
       <c r="A48" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="B48" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="C48" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
     </row>
     <row r="49" spans="1:3">
       <c r="A49" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="B49" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="C49" t="s">
         <v>202</v>
@@ -8105,10 +8168,10 @@
     </row>
     <row r="50" spans="1:3">
       <c r="A50" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="B50" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="C50" t="s">
         <v>202</v>
@@ -8116,10 +8179,10 @@
     </row>
     <row r="51" spans="1:3">
       <c r="A51" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="B51" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="C51" t="s">
         <v>202</v>
@@ -8127,10 +8190,10 @@
     </row>
     <row r="52" spans="1:3">
       <c r="A52" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="B52" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="C52" t="s">
         <v>202</v>
@@ -8138,21 +8201,21 @@
     </row>
     <row r="53" spans="1:3">
       <c r="A53" t="s">
+        <v>299</v>
+      </c>
+      <c r="B53" t="s">
+        <v>300</v>
+      </c>
+      <c r="C53" t="s">
         <v>301</v>
-      </c>
-      <c r="B53" t="s">
-        <v>302</v>
-      </c>
-      <c r="C53" t="s">
-        <v>202</v>
       </c>
     </row>
     <row r="54" spans="1:3">
       <c r="A54" t="s">
+        <v>302</v>
+      </c>
+      <c r="B54" t="s">
         <v>303</v>
-      </c>
-      <c r="B54" t="s">
-        <v>304</v>
       </c>
       <c r="C54" t="s">
         <v>202</v>
@@ -8160,10 +8223,10 @@
     </row>
     <row r="55" spans="1:3">
       <c r="A55" t="s">
+        <v>304</v>
+      </c>
+      <c r="B55" t="s">
         <v>305</v>
-      </c>
-      <c r="B55" t="s">
-        <v>306</v>
       </c>
       <c r="C55" t="s">
         <v>202</v>
@@ -8171,13 +8234,13 @@
     </row>
     <row r="56" spans="1:3">
       <c r="A56" t="s">
+        <v>306</v>
+      </c>
+      <c r="B56" t="s">
         <v>307</v>
       </c>
-      <c r="B56" t="s">
-        <v>265</v>
-      </c>
       <c r="C56" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
     </row>
     <row r="57" spans="1:3">
@@ -8185,7 +8248,7 @@
         <v>308</v>
       </c>
       <c r="B57" t="s">
-        <v>230</v>
+        <v>309</v>
       </c>
       <c r="C57" t="s">
         <v>202</v>
@@ -8193,10 +8256,10 @@
     </row>
     <row r="58" spans="1:3">
       <c r="A58" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="B58" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C58" t="s">
         <v>202</v>
@@ -8204,10 +8267,10 @@
     </row>
     <row r="59" spans="1:3">
       <c r="A59" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="B59" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="C59" t="s">
         <v>202</v>
@@ -8215,10 +8278,10 @@
     </row>
     <row r="60" spans="1:3">
       <c r="A60" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="B60" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="C60" t="s">
         <v>202</v>
@@ -8226,12 +8289,133 @@
     </row>
     <row r="61" spans="1:3">
       <c r="A61" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="B61" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C61" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3">
+      <c r="A62" t="s">
+        <v>318</v>
+      </c>
+      <c r="B62" t="s">
+        <v>319</v>
+      </c>
+      <c r="C62" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3">
+      <c r="A63" t="s">
+        <v>320</v>
+      </c>
+      <c r="B63" t="s">
+        <v>321</v>
+      </c>
+      <c r="C63" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3">
+      <c r="A64" t="s">
+        <v>322</v>
+      </c>
+      <c r="B64" t="s">
+        <v>278</v>
+      </c>
+      <c r="C64" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3">
+      <c r="A65" t="s">
+        <v>323</v>
+      </c>
+      <c r="B65" t="s">
+        <v>230</v>
+      </c>
+      <c r="C65" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3">
+      <c r="A66" t="s">
+        <v>324</v>
+      </c>
+      <c r="B66" t="s">
+        <v>325</v>
+      </c>
+      <c r="C66" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3">
+      <c r="A67" t="s">
+        <v>326</v>
+      </c>
+      <c r="B67" t="s">
+        <v>327</v>
+      </c>
+      <c r="C67" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3">
+      <c r="A68" t="s">
+        <v>328</v>
+      </c>
+      <c r="B68" t="s">
+        <v>329</v>
+      </c>
+      <c r="C68" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3">
+      <c r="A69" t="s">
+        <v>330</v>
+      </c>
+      <c r="B69" t="s">
+        <v>331</v>
+      </c>
+      <c r="C69" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3">
+      <c r="A70" t="s">
+        <v>332</v>
+      </c>
+      <c r="B70" t="s">
+        <v>333</v>
+      </c>
+      <c r="C70" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3">
+      <c r="A71" t="s">
+        <v>334</v>
+      </c>
+      <c r="B71" t="s">
+        <v>335</v>
+      </c>
+      <c r="C71" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3">
+      <c r="A72" t="s">
+        <v>336</v>
+      </c>
+      <c r="B72" t="s">
+        <v>337</v>
+      </c>
+      <c r="C72" t="s">
         <v>202</v>
       </c>
     </row>

</xml_diff>